<commit_message>
Tennis pipeline 2026-06-14: 5 articles, 18 social posts, triple finals Sunday
Stories: Stuttgart all-American final (Fritz vs Shelton, first in 71 years),
Queen's Club WTA final (Raducanu vs Vekic, British history on the line),
Libema Open final (Majchrzak Cinderella vs de Minaur), Wimbledon 15-day
preview, Triple Finals Sunday grass recap. PostPlanner: 18 posts (8 X + 10
FB) + 13 TOBI. WordPress blocked (environment restriction, known issue).
</commit_message>
<xml_diff>
--- a/Tennis/postplanner-imports/tfr-postplanner-2026-06-13.xlsx
+++ b/Tennis/postplanner-imports/tfr-postplanner-2026-06-13.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/13/2026  12:53</t>
+          <t>06/13/2026  08:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,7 +490,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06/13/2026  14:01</t>
+          <t>06/13/2026  10:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06/13/2026  15:09</t>
+          <t>06/13/2026  10:35</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06/13/2026  16:17</t>
+          <t>06/13/2026  12:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -526,7 +526,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/13/2026  17:25</t>
+          <t>06/13/2026  12:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -538,7 +538,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/13/2026  18:33</t>
+          <t>06/13/2026  15:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06/13/2026  19:41</t>
+          <t>06/13/2026  18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06/13/2026  20:49</t>
+          <t>06/13/2026  21:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>